<commit_message>
AMPLIA SRI-REPORTE DE VENTAS ALEX
</commit_message>
<xml_diff>
--- a/addons/account_ats/reports/reporte_ventas.xlsx
+++ b/addons/account_ats/reports/reporte_ventas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eduardo\eclipse-workspace\odoo16\addons16\pas_addons\pas_electronic_documents_ec_ats\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\sistemas\odoo_galarplan_project\addons\addons\account_ats\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3847C2F0-59B0-4450-B748-37B7DC8FA052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0712E318-954E-4977-87A4-0F9434762A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REPORTE DE VENTAS" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t># LINEAS:</t>
   </si>
@@ -92,6 +92,24 @@
   </si>
   <si>
     <t>Motivo Anulacion</t>
+  </si>
+  <si>
+    <t>¿Es vehículo?</t>
+  </si>
+  <si>
+    <t>Asesor</t>
+  </si>
+  <si>
+    <t>Estado Pago</t>
+  </si>
+  <si>
+    <t>Campo</t>
+  </si>
+  <si>
+    <t>Descripcion</t>
+  </si>
+  <si>
+    <t>Doc. Afectado NC</t>
   </si>
 </sst>
 </file>
@@ -553,16 +571,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="23.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Y4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="23.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.85546875" style="1"/>
-    <col min="5" max="6" width="23.85546875" style="2"/>
-    <col min="9" max="12" width="23.85546875" style="2"/>
-    <col min="14" max="14" width="23.85546875" style="2"/>
+    <col min="2" max="2" width="23.88671875" style="1"/>
+    <col min="5" max="6" width="23.88671875" style="2"/>
+    <col min="9" max="12" width="23.88671875" style="2"/>
+    <col min="14" max="14" width="23.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="8" customFormat="1" ht="30" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:25" s="8" customFormat="1" ht="29.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="11"/>
       <c r="B1" s="11"/>
       <c r="C1" s="11" t="s">
@@ -579,7 +597,7 @@
       <c r="L1" s="10"/>
       <c r="N1" s="9"/>
     </row>
-    <row r="2" spans="1:19" ht="18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
@@ -597,7 +615,7 @@
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
     </row>
-    <row r="3" spans="1:19" ht="18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
@@ -613,7 +631,7 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>1</v>
       </c>
@@ -670,6 +688,24 @@
       </c>
       <c r="S4" s="7" t="s">
         <v>15</v>
+      </c>
+      <c r="T4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="U4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="V4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="W4" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="X4" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y4" s="7" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>